<commit_message>
update manual armor disturbance experiment for SI
</commit_message>
<xml_diff>
--- a/experiments/armor_removal_experiment/Experiment_Summer2021.xlsx
+++ b/experiments/armor_removal_experiment/Experiment_Summer2021.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\hysteresis\experiments\armor_removal_experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F926A568-F551-4281-8F45-F9C54FBEB5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C394D13-FE17-4A32-8391-6BF29FE5C4F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{FA091B27-2BB3-44B8-A3BE-335E370FA65E}"/>
   </bookViews>
@@ -211,17 +211,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -262,32 +262,42 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx2"/>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="es-AR"/>
+              <a:rPr lang="es-AR" b="0" i="0">
+                <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
               <a:t>Experimental</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="es-AR" baseline="0"/>
+              <a:rPr lang="es-AR" b="0" i="0" baseline="0">
+                <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
               <a:t> c</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="es-AR"/>
+              <a:rPr lang="es-AR" b="0" i="0">
+                <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
               <a:t>onstituent</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="es-AR" baseline="0"/>
+              <a:rPr lang="es-AR" b="0" i="0" baseline="0">
+                <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
               <a:t> concentrations </a:t>
             </a:r>
-            <a:endParaRPr lang="es-AR"/>
+            <a:endParaRPr lang="es-AR" b="0" i="0">
+              <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -304,11 +314,11 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx2"/>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
@@ -438,7 +448,7 @@
             <c:numRef>
               <c:f>Sheet1!$D$3:$D$18</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>3.4553255204584259</c:v>
@@ -613,7 +623,7 @@
             <c:numRef>
               <c:f>Sheet1!$E$3:$E$18</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>1.1019061775871011</c:v>
@@ -1048,7 +1058,7 @@
           <c:idx val="3"/>
           <c:order val="3"/>
           <c:tx>
-            <c:v>TP</c:v>
+            <c:v>PP</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="9525" cap="rnd">
@@ -1164,57 +1174,57 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$I$3:$I$18</c:f>
+              <c:f>Sheet1!$G$3:$G$18</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
-                  <c:v>0.03</c:v>
+                  <c:v>5.1576641217063925E-5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.9E-2</c:v>
+                  <c:v>2.9040962645844913E-4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.5999999999999999E-2</c:v>
+                  <c:v>6.6106276627512963E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.1999999999999995E-2</c:v>
+                  <c:v>2.2224172067829232E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.1000000000000003E-2</c:v>
+                  <c:v>2.0552078586848492E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.11799999999999999</c:v>
+                  <c:v>2.3927254516111322E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.05</c:v>
+                  <c:v>2.5382950090458741E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.3000000000000002E-2</c:v>
+                  <c:v>3.8420401139033575E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.03</c:v>
+                  <c:v>4.6887855651876298E-5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.7E-2</c:v>
+                  <c:v>1.2779120936401461E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.7E-2</c:v>
+                  <c:v>4.4474966741118462E-6</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.5999999999999999E-2</c:v>
+                  <c:v>4.6887855651876298E-5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.1E-2</c:v>
+                  <c:v>1.4986210786444661E-4</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.4E-2</c:v>
+                  <c:v>5.1576641217063925E-5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2.5000000000000001E-2</c:v>
+                  <c:v>4.8981773007164672E-4</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.03</c:v>
+                  <c:v>4.9120610682918029E-5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1269,13 +1279,15 @@
                     <a:solidFill>
                       <a:schemeClr val="tx2"/>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="es-AR"/>
+                  <a:rPr lang="es-AR">
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
                   <a:t>Time elapsed</a:t>
                 </a:r>
               </a:p>
@@ -1298,7 +1310,7 @@
                   <a:solidFill>
                     <a:schemeClr val="tx2"/>
                   </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
+                  <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
@@ -1379,20 +1391,26 @@
                     <a:solidFill>
                       <a:schemeClr val="tx2"/>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="es-AR"/>
+                  <a:rPr lang="es-AR">
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
                   <a:t>POC, DOC</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="es-AR" baseline="0"/>
+                  <a:rPr lang="es-AR" baseline="0">
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
                   <a:t> and SS (mg/L)</a:t>
                 </a:r>
-                <a:endParaRPr lang="es-AR"/>
+                <a:endParaRPr lang="es-AR">
+                  <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+                </a:endParaRPr>
               </a:p>
             </c:rich>
           </c:tx>
@@ -1413,7 +1431,7 @@
                   <a:solidFill>
                     <a:schemeClr val="tx2"/>
                   </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
+                  <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
@@ -1462,6 +1480,7 @@
       <c:valAx>
         <c:axId val="1879921696"/>
         <c:scaling>
+          <c:logBase val="10"/>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -1477,20 +1496,26 @@
                     <a:solidFill>
                       <a:schemeClr val="tx2"/>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="es-AR"/>
-                  <a:t>SRP and TP</a:t>
+                  <a:rPr lang="es-AR">
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
+                  <a:t>SRP and PP</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="es-AR" baseline="0"/>
+                  <a:rPr lang="es-AR" baseline="0">
+                    <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
                   <a:t> (mg/L)</a:t>
                 </a:r>
-                <a:endParaRPr lang="es-AR"/>
+                <a:endParaRPr lang="es-AR">
+                  <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
+                </a:endParaRPr>
               </a:p>
             </c:rich>
           </c:tx>
@@ -1511,7 +1536,7 @@
                   <a:solidFill>
                     <a:schemeClr val="tx2"/>
                   </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
+                  <a:latin typeface="Abadi" panose="020B0604020104020204" pitchFamily="34" charset="0"/>
                   <a:ea typeface="+mn-ea"/>
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
@@ -1811,7 +1836,7 @@
             <c:numRef>
               <c:f>Sheet1!$D$3:$D$18</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>3.4553255204584259</c:v>
@@ -1868,7 +1893,7 @@
             <c:numRef>
               <c:f>Sheet1!$E$3:$E$18</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>1.1019061775871011</c:v>
@@ -2020,7 +2045,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2137,7 +2162,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2389,7 +2414,7 @@
             <c:numRef>
               <c:f>Sheet1!$D$3:$D$18</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>3.4553255204584259</c:v>
@@ -2598,7 +2623,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2967,7 +2992,7 @@
             <c:numRef>
               <c:f>Sheet1!$D$3:$D$18</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>3.4553255204584259</c:v>
@@ -3176,7 +3201,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3545,7 +3570,7 @@
             <c:numRef>
               <c:f>Sheet1!$D$3:$D$18</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>3.4553255204584259</c:v>
@@ -3754,7 +3779,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -7927,6 +7952,7 @@
   <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
     <col min="3" max="3" width="17.42578125" customWidth="1"/>
     <col min="4" max="4" width="18.5703125" customWidth="1"/>
     <col min="5" max="5" width="17.28515625" customWidth="1"/>
@@ -7937,31 +7963,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D1" s="7">
+      <c r="D1" s="5">
         <f>MAX(D3:D18)</f>
         <v>240.0916933100078</v>
       </c>
-      <c r="E1" s="7">
+      <c r="E1" s="5">
         <f t="shared" ref="E1:J1" si="0">MAX(E3:E18)</f>
         <v>38.658748032082826</v>
       </c>
-      <c r="F1" s="7">
+      <c r="F1" s="5">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="G1" s="7">
+      <c r="G1" s="5">
         <f t="shared" si="0"/>
         <v>2.3927254516111322E-3</v>
       </c>
-      <c r="H1" s="7">
+      <c r="H1" s="5">
         <f t="shared" si="0"/>
         <v>2.4E-2</v>
       </c>
-      <c r="I1" s="7">
+      <c r="I1" s="5">
         <f t="shared" si="0"/>
         <v>0.11799999999999999</v>
       </c>
-      <c r="J1" s="7">
+      <c r="J1" s="5">
         <f t="shared" si="0"/>
         <v>2.1269999999999998</v>
       </c>
@@ -8008,7 +8034,7 @@
       <c r="C3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="7">
         <v>3.4553255204584259</v>
       </c>
       <c r="E3" s="4">
@@ -8017,7 +8043,7 @@
       <c r="F3" s="1">
         <v>0</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="8">
         <v>5.1576641217063925E-5</v>
       </c>
       <c r="H3" s="1">
@@ -8026,7 +8052,7 @@
       <c r="I3" s="1">
         <v>0.03</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="4">
         <v>2.1269999999999998</v>
       </c>
     </row>
@@ -8041,7 +8067,7 @@
       <c r="C4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="7">
         <v>19.697185438321707</v>
       </c>
       <c r="E4" s="4">
@@ -8050,7 +8076,7 @@
       <c r="F4" s="1">
         <v>3</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="8">
         <v>2.9040962645844913E-4</v>
       </c>
       <c r="H4" s="1">
@@ -8059,7 +8085,7 @@
       <c r="I4" s="1">
         <v>3.9E-2</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="4">
         <v>1.3859999999999999</v>
       </c>
     </row>
@@ -8074,7 +8100,7 @@
       <c r="C5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <v>52.651576833306279</v>
       </c>
       <c r="E5" s="4">
@@ -8084,7 +8110,7 @@
         <f>F4+3</f>
         <v>6</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="8">
         <v>6.6106276627512963E-4</v>
       </c>
       <c r="H5" s="1">
@@ -8093,7 +8119,7 @@
       <c r="I5" s="1">
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="4">
         <v>1.5820000000000001</v>
       </c>
     </row>
@@ -8108,7 +8134,7 @@
       <c r="C6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <v>89.933968747198861</v>
       </c>
       <c r="E6" s="4">
@@ -8118,7 +8144,7 @@
         <f t="shared" ref="F6:F18" si="2">F5+3</f>
         <v>9</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="8">
         <v>2.2224172067829232E-3</v>
       </c>
       <c r="H6" s="1">
@@ -8127,7 +8153,7 @@
       <c r="I6" s="1">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="4">
         <v>1.643</v>
       </c>
     </row>
@@ -8142,7 +8168,7 @@
       <c r="C7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <v>73.619940199502565</v>
       </c>
       <c r="E7" s="4">
@@ -8152,7 +8178,7 @@
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="8">
         <v>2.0552078586848492E-3</v>
       </c>
       <c r="H7" s="1">
@@ -8161,7 +8187,7 @@
       <c r="I7" s="1">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="4">
         <v>1.5389999999999999</v>
       </c>
     </row>
@@ -8176,7 +8202,7 @@
       <c r="C8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <v>240.0916933100078</v>
       </c>
       <c r="E8" s="4">
@@ -8186,7 +8212,7 @@
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="8">
         <v>2.3927254516111322E-3</v>
       </c>
       <c r="H8" s="1">
@@ -8195,7 +8221,7 @@
       <c r="I8" s="1">
         <v>0.11799999999999999</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="4">
         <v>1.502</v>
       </c>
     </row>
@@ -8210,7 +8236,7 @@
       <c r="C9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="7">
         <v>73.574494175352541</v>
       </c>
       <c r="E9" s="4">
@@ -8220,7 +8246,7 @@
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="8">
         <v>2.5382950090458741E-4</v>
       </c>
       <c r="H9" s="1">
@@ -8229,7 +8255,7 @@
       <c r="I9" s="1">
         <v>0.05</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <v>1.46</v>
       </c>
     </row>
@@ -8244,7 +8270,7 @@
       <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="7">
         <v>20.816385127051692</v>
       </c>
       <c r="E10" s="4">
@@ -8254,7 +8280,7 @@
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="8">
         <v>3.8420401139033575E-4</v>
       </c>
       <c r="H10" s="1">
@@ -8263,7 +8289,7 @@
       <c r="I10" s="1">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="4">
         <v>1.4370000000000001</v>
       </c>
     </row>
@@ -8278,7 +8304,7 @@
       <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="7">
         <v>17.667101333445487</v>
       </c>
       <c r="E11" s="4">
@@ -8288,7 +8314,7 @@
         <f t="shared" si="2"/>
         <v>24</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="8">
         <v>4.6887855651876298E-5</v>
       </c>
       <c r="H11" s="1">
@@ -8297,7 +8323,7 @@
       <c r="I11" s="1">
         <v>0.03</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="4">
         <v>1.6559999999999999</v>
       </c>
     </row>
@@ -8312,7 +8338,7 @@
       <c r="C12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="7">
         <v>15.963635379745167</v>
       </c>
       <c r="E12" s="4">
@@ -8322,7 +8348,7 @@
         <f t="shared" si="2"/>
         <v>27</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="8">
         <v>1.2779120936401461E-4</v>
       </c>
       <c r="H12" s="1">
@@ -8331,7 +8357,7 @@
       <c r="I12" s="1">
         <v>2.7E-2</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="4">
         <v>1.7370000000000001</v>
       </c>
     </row>
@@ -8346,7 +8372,7 @@
       <c r="C13" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="7">
         <v>7.0668603509873824</v>
       </c>
       <c r="E13" s="4">
@@ -8356,7 +8382,7 @@
         <f t="shared" si="2"/>
         <v>30</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="8">
         <v>4.4474966741118462E-6</v>
       </c>
       <c r="H13" s="1">
@@ -8365,7 +8391,7 @@
       <c r="I13" s="1">
         <v>2.7E-2</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="4">
         <v>1.4590000000000001</v>
       </c>
     </row>
@@ -8380,7 +8406,7 @@
       <c r="C14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="7">
         <v>12.436951564983044</v>
       </c>
       <c r="E14" s="4">
@@ -8390,7 +8416,7 @@
         <f t="shared" si="2"/>
         <v>33</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="8">
         <v>4.6887855651876298E-5</v>
       </c>
       <c r="H14" s="1">
@@ -8399,7 +8425,7 @@
       <c r="I14" s="1">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="4">
         <v>1.6379999999999999</v>
       </c>
     </row>
@@ -8414,7 +8440,7 @@
       <c r="C15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="7">
         <v>8.095527221210272</v>
       </c>
       <c r="E15" s="4">
@@ -8424,7 +8450,7 @@
         <f t="shared" si="2"/>
         <v>36</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15" s="8">
         <v>1.4986210786444661E-4</v>
       </c>
       <c r="H15" s="1">
@@ -8433,7 +8459,7 @@
       <c r="I15" s="1">
         <v>3.1E-2</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="4">
         <v>1.7050000000000001</v>
       </c>
     </row>
@@ -8448,7 +8474,7 @@
       <c r="C16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="7">
         <v>10.855405992184116</v>
       </c>
       <c r="E16" s="4">
@@ -8458,7 +8484,7 @@
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16" s="8">
         <v>5.1576641217063925E-5</v>
       </c>
       <c r="H16" s="1">
@@ -8467,7 +8493,7 @@
       <c r="I16" s="1">
         <v>2.4E-2</v>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="4">
         <v>1.7070000000000001</v>
       </c>
     </row>
@@ -8482,7 +8508,7 @@
       <c r="C17" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="7">
         <v>6.0885448377837434</v>
       </c>
       <c r="E17" s="4">
@@ -8492,7 +8518,7 @@
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
-      <c r="G17" s="1">
+      <c r="G17" s="8">
         <v>4.8981773007164672E-4</v>
       </c>
       <c r="H17" s="1">
@@ -8501,7 +8527,7 @@
       <c r="I17" s="1">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="4">
         <v>1.681</v>
       </c>
     </row>
@@ -8516,7 +8542,7 @@
       <c r="C18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="7">
         <v>11.464181780769531</v>
       </c>
       <c r="E18" s="4">
@@ -8526,7 +8552,7 @@
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="G18" s="1">
+      <c r="G18" s="8">
         <v>4.9120610682918029E-5</v>
       </c>
       <c r="H18" s="1">
@@ -8535,26 +8561,26 @@
       <c r="I18" s="1">
         <v>0.03</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="4">
         <v>1.262</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D19" s="7">
+      <c r="D19" s="5">
         <f>AVERAGE(D12:D18)</f>
         <v>10.281586732523323</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="5">
         <f>AVERAGE(E13:E18)</f>
         <v>2.3721951057441486</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>